<commit_message>
Deploying to gh-pages from  @ e5a583deed6ab0f8cdfc75849cb2c7e54039e294 🚀
</commit_message>
<xml_diff>
--- a/en/downloads/data-excel/10.3.1.1.xlsx
+++ b/en/downloads/data-excel/10.3.1.1.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17801D1E-0BAC-47A1-9A91-DDE256C7C62D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -16,15 +17,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
-    <t>10.3.1.1а Анын ичинде каралган жана канааттандырылган Омбудсменге кайрылуулардын саны</t>
-  </si>
-  <si>
-    <t>10.3.1.1а Количество обращений к Омбудсмену, из них рассмотренных и удовлетворенных</t>
-  </si>
-  <si>
-    <t>10.3.1.1a Number of appeals to the Ombudsman, of which examined and satisfied</t>
-  </si>
-  <si>
     <t>Көрсөткүчтөрдүн аталышы</t>
   </si>
   <si>
@@ -53,18 +45,35 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>10.3.1.1 Количество обращений к Омбудсмену, из них рассмотренных и удовлетворенных</t>
+  </si>
+  <si>
+    <t>10.3.1.1 Number of appeals to the Ombudsman, of which examined and satisfied</t>
+  </si>
+  <si>
+    <t>10.3.1.1 Анын ичинде каралган жана канааттандырылган Омбудсменге кайрылуулардын саны</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -124,35 +133,40 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный 2" xfId="1" xr:uid="{072C404C-4BA3-4539-91CA-34107B947B1F}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -168,9 +182,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -208,9 +222,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -245,7 +259,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -280,7 +294,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -453,22 +467,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:U5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="36.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -485,7 +499,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -506,16 +520,17 @@
       <c r="R2" s="3"/>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
+      <c r="U2" s="11"/>
     </row>
-    <row r="3" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3" s="5">
         <v>2007</v>
@@ -568,16 +583,19 @@
       <c r="T3" s="6">
         <v>2023</v>
       </c>
+      <c r="U3" s="12">
+        <v>2024</v>
+      </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4" s="2">
         <v>3014</v>
@@ -630,25 +648,28 @@
       <c r="T4" s="7">
         <v>2620</v>
       </c>
+      <c r="U4" s="10">
+        <v>2663</v>
+      </c>
     </row>
-    <row r="5" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D5" s="3">
         <v>619</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G5" s="3">
         <v>309</v>
@@ -663,7 +684,7 @@
         <v>384</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="L5" s="3">
         <v>374</v>
@@ -691,6 +712,9 @@
       </c>
       <c r="T5" s="9">
         <v>264</v>
+      </c>
+      <c r="U5" s="11">
+        <v>780</v>
       </c>
     </row>
   </sheetData>

</xml_diff>